<commit_message>
doc: delete unnecessary QR-code text in Spaltenanalyse_Lieferantenabfrage.xlsx cell D41
</commit_message>
<xml_diff>
--- a/Meilenstein 1/Spaltenanalyse_Lieferantenabfrage.xlsx
+++ b/Meilenstein 1/Spaltenanalyse_Lieferantenabfrage.xlsx
@@ -1100,11 +1100,7 @@
           <t>Technische und grafische Anforderungen</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Der QR-Code auf dem grünen Label selbst wird vom Tool automatisch generiert (Verweis auf das EU-Portal 'Your Europe'). Vom Lieferanten wird in dieser Spalte ausschließlich der Link (URL) oder das PDF zu den herstellereigenen, detaillierten Garantiebedingungen benötigt.</t>
-        </is>
-      </c>
+      <c r="D41" s="5" t="n"/>
     </row>
     <row r="42" ht="63.75" customHeight="1" s="9">
       <c r="A42" s="3" t="inlineStr">

</xml_diff>

<commit_message>
doc: commit user edits in Spaltenanalyse_Lieferantenabfrage.xlsx (removed Spalte 5 Artikelbezeichnung, renumbered subsequent columns)
</commit_message>
<xml_diff>
--- a/Meilenstein 1/Spaltenanalyse_Lieferantenabfrage.xlsx
+++ b/Meilenstein 1/Spaltenanalyse_Lieferantenabfrage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thomas.winkler\Desktop\Projekte\Google Antigravity\ELEKTROPEPI\GEWAEHRLEISTUNG_GARANTIELABEL\Meilenstein 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A2A85F-1579-4FFC-9129-E34C0369F3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F954B4-DD5E-43BA-9B62-FF08125B353E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
   <si>
     <t>Spaltenanalyse für die Lieferanten-Garantieabfrage (EU 2025/1960)</t>
   </si>
@@ -120,27 +120,6 @@
     <t>Sehr gering.</t>
   </si>
   <si>
-    <t>Spalte 5: Artikelbezeichnung</t>
-  </si>
-  <si>
-    <t>Verzichtbar (Optional)</t>
-  </si>
-  <si>
-    <t>Für das Label gesetzlich nicht erforderlich (dort stehen nur Marke und Modellkennung).</t>
-  </si>
-  <si>
-    <t>Dient nur der manuellen Qualitätskontrolle beim Import. Wird nicht in Magento importiert, da wir eigene Bezeichnungen nutzen.</t>
-  </si>
-  <si>
-    <t>Höher (längerer Text zum Eintippen).</t>
-  </si>
-  <si>
-    <t>Kann weggelassen werden (reduziert den Aufwand für den Lieferanten).</t>
-  </si>
-  <si>
-    <t>Spalte 6: Garantiedauer in Jahren (XX)</t>
-  </si>
-  <si>
     <t>Angepasst werden muss:
 'XX' → wird ersetzt durch die Anzahl der Garantie-Jahre</t>
   </si>
@@ -151,13 +130,7 @@
     <t>Sehr gering (Eingabe einer Ganzzahl &gt; 2).</t>
   </si>
   <si>
-    <t>Spalte 7: Link zu den Garantiebedingungen</t>
-  </si>
-  <si>
     <t>Gesetzliche Pflicht zur Bereitstellung der Garantieerklärung für den Endkunden. Wird im Shop verlinkt (bzw. für Globus in m.PIM hochgeladen).</t>
-  </si>
-  <si>
-    <t>Spalte 8: Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)</t>
   </si>
   <si>
     <t>Dringend empfohlen zur Risiko-Vermeidung</t>
@@ -180,6 +153,15 @@
   </si>
   <si>
     <t>Gering (Eingabe einer Web-URL zu einer PDF oder Zusendung als PDF).</t>
+  </si>
+  <si>
+    <t>Spalte 5: Garantiedauer in Jahren (XX)</t>
+  </si>
+  <si>
+    <t>Spalte 6: Link zu den Garantiebedingungen</t>
+  </si>
+  <si>
+    <t>Spalte 7: Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)</t>
   </si>
 </sst>
 </file>
@@ -659,7 +641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -905,7 +887,7 @@
     <row r="27" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -916,21 +898,21 @@
         <v>6</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
@@ -940,7 +922,7 @@
         <v>12</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
@@ -950,7 +932,7 @@
         <v>14</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
@@ -958,7 +940,7 @@
     <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -972,28 +954,28 @@
         <v>22</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
     </row>
-    <row r="37" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
@@ -1011,7 +993,7 @@
     <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B40" s="9"/>
       <c r="C40" s="9"/>
@@ -1022,31 +1004,31 @@
         <v>6</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
     </row>
-    <row r="43" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
@@ -1062,86 +1044,30 @@
       <c r="D44" s="7"/>
     </row>
     <row r="45" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="10"/>
-    </row>
-    <row r="47" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-    </row>
-    <row r="49" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-    </row>
-    <row r="50" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-    </row>
-    <row r="51" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="C47:C50"/>
+  <mergeCells count="22">
+    <mergeCell ref="C41:C44"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="D35:D38"/>
+    <mergeCell ref="C17:C20"/>
     <mergeCell ref="D41:D44"/>
-    <mergeCell ref="C17:C20"/>
-    <mergeCell ref="D47:D50"/>
     <mergeCell ref="C11:C14"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="C23:C26"/>
-    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="D5:D8"/>
     <mergeCell ref="D23:D26"/>
-    <mergeCell ref="D35:D38"/>
     <mergeCell ref="D29:D32"/>
-    <mergeCell ref="C41:C44"/>
     <mergeCell ref="C35:C38"/>
-    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="C29:C32"/>
+    <mergeCell ref="A34:D34"/>
     <mergeCell ref="D17:D20"/>
-    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="C5:C8"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="C29:C32"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="D11:D14"/>
-    <mergeCell ref="A28:D28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>